<commit_message>
minor enhancement null check for website and phone
</commit_message>
<xml_diff>
--- a/assets/temp-good.xlsx
+++ b/assets/temp-good.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="23530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="23628"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jared\source\repos\avtopia\data_sync_desktop\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2DF01ACB-60F7-4B82-A5F2-7E29C2F2D104}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C17D9B7D-0571-4AD1-8B12-AD087E890E6F}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,6 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Sheet2!$A$1:$M$263</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -17959,8 +17958,8 @@
   <cols>
     <col min="1" max="1" width="0" style="3" hidden="1" customWidth="1"/>
     <col min="2" max="2" width="31.125" style="24" customWidth="1"/>
-    <col min="3" max="3" width="23.5" style="3" hidden="1" customWidth="1"/>
-    <col min="4" max="5" width="12.5" style="3" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="23.5" style="3" customWidth="1"/>
+    <col min="4" max="5" width="12.5" style="3" customWidth="1"/>
     <col min="6" max="6" width="26.25" style="3" customWidth="1"/>
     <col min="7" max="7" width="29" style="3" customWidth="1"/>
     <col min="8" max="8" width="13.625" style="3" customWidth="1"/>

</xml_diff>